<commit_message>
Added google-genai model class
</commit_message>
<xml_diff>
--- a/data/dataset_complete(Data Scientist).xlsx
+++ b/data/dataset_complete(Data Scientist).xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,21 +413,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>JD</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Resume</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Response</t>
         </is>
@@ -13420,6 +13408,346 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Requirements
+ Description and Requirements 
+Title: Data Partner - Computer Science
+Location: Asia - Remote
+Are you ready to use your domain knowledge to advance AI? Join us as a Data Partner and work remotely with flexible hours. We are seeking highly knowledgeable Subject Matter Expert to design advanced, domain-specific questions and solutions. The role involves creating challenging problem sets that test deep reasoning and expertise in the assigned field.
+Key Responsibilities:
+Develop complex, original question-and-answer pairs based on advanced topics in your area of expertise.
+Ensure questions involve multi-step problem-solving and critical thinking.
+Provide detailed, clear solutions that meet high academic standards.
+Collaborate with cross-functional teams to refine and enhance content.
+Basic Requirements:
+A completed master's degree, bachelor's degree, associate's degree or anything equivalent in Computer Science is essential
+Strong proficiency in English writing with excellent grammar, clarity, and the ability to explain complex concepts concisely
+Assessment:
+In order to be hired into the program, you’ll go through a subject-specific qualification exam that will determine your suitability for the position and complete ID verification.
+Payment:
+Currently, pay rates for experts range from $8 - $30 USD per hour
+Rates vary based on expertise, skills assessment, location, project need, and other factors. For example, higher rates may be offered to PhDs. Please review the payment terms for each project.
+Equal Opportunity:
+All qualified applicants will receive consideration for a contractual relationship without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, disability, or protected veteran status. At TELUS Digital AI, we are proud to offer equal opportunities and are committed to creating a diverse and inclusive community. All aspects of selection are based on applicants’ qualifications, merits, competence, and performance without regard to any characteristic related to diversity.
+Additional Job Description
+TELUS Digital AI Community
+Our global AI Community is a vibrant network of 1 million+ contributors from diverse backgrounds who help our customers collect, enhance, train, translate, and localize content to build better AI models. Become part of our growing community and make an impact supporting the machine learning models of some of the world’s largest brands.
+EEO Statement
+At TELUS International, we enable customer experience innovation through spirited teamwork, agile thinking, and a caring culture that puts customers first. TELUS International is the global arm of TELUS Corporation, one of the largest telecommunications service providers in Canada. We deliver contact center and business process outsourcing (BPO) solutions to some of the world's largest corporations in the consumer electronics, finance, telecommunications and utilities sectors. With global call center delivery capabilities, our multi-shore, multi-language programs offer safe, secure infrastructure, value-based pricing, skills-based resources and exceptional customer service - all backed by TELUS, our multi-billion dollar telecommunications parent.
+Equal Opportunity Employer
+At TELUS International, we are proud to be an equal opportunity employer and are committed to creating a diverse and inclusive workplace. All aspects of employment, including the decision to hire and promote, are based on applicants’ qualifications, merits, competence and performance without regard to any characteristic related to diversity.</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KEY SKILLS: Ã¢Â€Â¢ Planning &amp; Strategizing Ã¢Â€Â¢ Presentation skill Ã¢Â€Â¢ Client relationship Ã¢Â€Â¢ Energy level Ã¢Â€Â¢ Enquiry Generation Ã¢Â€Â¢ Achieving Targets QUALIFICATIONS: A university in marketing or business studies is preferred or a minimum of three years of related experience in sales &amp; marketing sector. Problem - solving and analytical skills to interpret sales performance and market trend information. Proven ability to motivate and lead the sales team. Experience in developing marketing and sales strategies. Excellent oral and written communication skills, plus a good working knowledge of Microsoft Office. Computer KNOWLEDGE Ã¢Â€Â¢ Knowledge of MS Excel, MS Word, MS PowerPoint achievements and Interests Ã¢Â€Â¢ I played Cricket for National Team (Maharashtra Cricket Association) Ã¢Â€Â¢ Played Regional level Cricket Tournament Thee times for School team Ã¢Â€Â¢ Worked as a Sports Secretary in college annual meet. Ã¢Â€Â¢ Worked as a volunteer for road show in POONA College. Ã¢Â€Â¢ Worked as a Group leader for college presentation. Ã¢Â€Â¢ My Interest are Learning various computers languages &amp; Tricks and Techniques of computer and Playing Cricket. personal Information . Education Details 
+ MBA Operations  Dr. D. Y. Patil College
+ B.B.A. Marketing Pune, Maharashtra Poona College
+ H. S. C.   Moledina high School &amp; Jr. College
+ S. S. C. Maharashtra Board  A.M.V.High School
+Sales manager 
+Sales Manager
+Skill Details 
+SALES- Exprience - 104 months
+MARKETING- Exprience - 97 months
+SALES TEAM- Exprience - 44 months
+AND SALES- Exprience - 6 months
+EXCEL- Exprience - 6 monthsCompany Details 
+company - F2 Fun Fitness
+description - Ã¢Â€Â¢	Set individual sales targets with sales team.
+Ã¢Â€Â¢	Handling Enquiries.
+Ã¢Â€Â¢	Generating new enquiries
+Ã¢Â€Â¢	Set individual sales targets with sales team.
+Ã¢Â€Â¢	Continuously managing team performance.Ã‚Â 
+Ã¢Â€Â¢	Managing staff training requirements.Ã‚Â 
+Ã‚Â 
+Ã¢Â€Â¢	Generate timely sales reports.
+Ã¢Â€Â¢	Organizing seasonal promotions and events.
+Ã¢Â€Â¢	Supervise and motivate staff.
+Ã¢Â€Â¢	Ã‚Â Ã‚Â Holds regular meeting with sales staff.
+company - Gold's Gym India Pvt Ltd
+description - JOB PROFILE:
+Ã¢Â€Â¢ Set individual sales targets with sales team.
+Ã¢Â€Â¢ Handling Enquiries.
+Ã¢Â€Â¢ Generating new enquiries
+Ã¢Â€Â¢ Set individual sales targets with sales team.
+Ã¢Â€Â¢ Continuously managing team performance.
+Ã¢Â€Â¢ Managing staff training requirements.
+Ã¢Â€Â¢ Generate timely sales reports.
+Ã¢Â€Â¢ Organizing seasonal promotions and events.
+Ã¢Â€Â¢ Supervise and motivate staff.
+Ã¢Â€Â¢ Holds regular meeting with sales staff.
+company - 
+description - 10 to 24/2012
+Achievements: Joined as a sales associate in 2010. Promoted to Sales Manager 2012.
+Exceeded sales targets with high level of contribution &amp; dedication to the organization.
+Applauded for Best sales &amp; marketing performance in Pune zone &amp; Awarded the
+Ã¢Â€Â¢    Certificate of Excellence &amp; outstanding performance in the year 2014. Ranked as #1 sales manager (out of 6) in 2013 and 2014. Recognized for superior performance as a two-time district "Employee of the Month" honoree.
+JOB PROFILE:
+Ã¢Â€Â¢ Build strategies and develop marketing initiative to create awareness of company services.
+Ã¢Â€Â¢ Propose and execute the promotional programme to attract clients.
+Ã¢Â€Â¢ Working with the team of four - six people thereby ensuring that targets defined are achieved.
+Ã¢Â€Â¢ Arrange all the necessary &amp; possible facilities for information desk.
+Ã¢Â€Â¢ Manages personal and develops sales roles support staff.
+Ã¢Â€Â¢ Reviews progress of sales roles throughout the company.
+Ã¢Â€Â¢ Determine price schedules and discount rate.
+Ã¢Â€Â¢ Generate timely sales reports.
+Ã¢Â€Â¢ Control expenses and monitor budgets.
+company - Talwalkars Aspire Fitness Pvt Ltd
+description - 
+company - Talwalkars Aspire Fitness Pvt Ltd
+description - </t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>```json
+{
+    "summary": "The candidate is an entirely mismatched fit for this role. The job description requires a Subject Matter Expert in Computer Science with a relevant degree to create complex technical content for AI training. The candidate's entire professional background and education are in Sales, Marketing, and Business Administration.",
+    "match_score": 5,
+    "skill_match": {
+        "matched": [
+            "English writing (implied via professional experience)"
+        ],
+        "missing": [
+            "Advanced Computer Science domain knowledge",
+            "Multi-step technical problem-solving",
+            "Ability to design complex CS question-and-answer pairs",
+            "Academic-standard technical writing"
+        ],
+        "score": 10
+    },
+    "experience_match": {
+        "matched_years": 0,
+        "required_years": "Not specified (requires subject matter expertise)",
+        "score": 0
+    },
+    "education_match": {
+        "matched_degree": "None",
+        "required_degree": "Bachelor's, Master's, or Associate's in Computer Science",
+        "score": 0
+    },
+    "responsibility_match": {
+        "matched": [],
+        "missing": [
+            "Developing complex, original Q&amp;A pairs in Computer Science",
+            "Creating problem sets that test deep reasoning",
+            "Providing detailed technical solutions",
+            "Collaborating on technical content refinement"
+        ],
+        "score": 0
+    },
+    "final_assessment": "Weak fit"
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Requirements
+ Description and Requirements 
+Title: Data Partner - Computer Science
+Location: Asia - Remote
+Are you ready to use your domain knowledge to advance AI? Join us as a Data Partner and work remotely with flexible hours. We are seeking highly knowledgeable Subject Matter Expert to design advanced, domain-specific questions and solutions. The role involves creating challenging problem sets that test deep reasoning and expertise in the assigned field.
+Key Responsibilities:
+Develop complex, original question-and-answer pairs based on advanced topics in your area of expertise.
+Ensure questions involve multi-step problem-solving and critical thinking.
+Provide detailed, clear solutions that meet high academic standards.
+Collaborate with cross-functional teams to refine and enhance content.
+Basic Requirements:
+A completed master's degree, bachelor's degree, associate's degree or anything equivalent in Computer Science is essential
+Strong proficiency in English writing with excellent grammar, clarity, and the ability to explain complex concepts concisely
+Assessment:
+In order to be hired into the program, you’ll go through a subject-specific qualification exam that will determine your suitability for the position and complete ID verification.
+Payment:
+Currently, pay rates for experts range from $8 - $30 USD per hour
+Rates vary based on expertise, skills assessment, location, project need, and other factors. For example, higher rates may be offered to PhDs. Please review the payment terms for each project.
+Equal Opportunity:
+All qualified applicants will receive consideration for a contractual relationship without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, disability, or protected veteran status. At TELUS Digital AI, we are proud to offer equal opportunities and are committed to creating a diverse and inclusive community. All aspects of selection are based on applicants’ qualifications, merits, competence, and performance without regard to any characteristic related to diversity.
+Additional Job Description
+TELUS Digital AI Community
+Our global AI Community is a vibrant network of 1 million+ contributors from diverse backgrounds who help our customers collect, enhance, train, translate, and localize content to build better AI models. Become part of our growing community and make an impact supporting the machine learning models of some of the world’s largest brands.
+EEO Statement
+At TELUS International, we enable customer experience innovation through spirited teamwork, agile thinking, and a caring culture that puts customers first. TELUS International is the global arm of TELUS Corporation, one of the largest telecommunications service providers in Canada. We deliver contact center and business process outsourcing (BPO) solutions to some of the world's largest corporations in the consumer electronics, finance, telecommunications and utilities sectors. With global call center delivery capabilities, our multi-shore, multi-language programs offer safe, secure infrastructure, value-based pricing, skills-based resources and exceptional customer service - all backed by TELUS, our multi-billion dollar telecommunications parent.
+Equal Opportunity Employer
+At TELUS International, we are proud to be an equal opportunity employer and are committed to creating a diverse and inclusive workplace. All aspects of employment, including the decision to hire and promote, are based on applicants’ qualifications, merits, competence and performance without regard to any characteristic related to diversity.</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>IT Skills: MS Office. Photoshop. SQL Server.Education Details 
+June 2015 Bachelor   Yashwantrao chavan maharashtra university
+Sales Manager 
+Sales Manager
+Skill Details 
+MS OFFICE- Exprience - 6 months
+MS SQL SERVER- Exprience - 6 months
+PHOTOSHOP- Exprience - 6 months
+SQL- Exprience - 6 months
+SQL SERVER- Exprience - 6 monthsCompany Details 
+company - Nature Of Work
+description - Generating leads on calls, Suggesting Residential property as per clients budget &amp; specification, building Relationship with Channel Partner.
+Ã¢ÂžÂ¢  Meeting with clients for project presentation follow for up Site Visit
+Deal closure.
+Worked with ICICI Merchant services (Hgs Payroll) As Sales Manager. (16th Jan 2017 to till 30th Aug 2018)
+Nature of Work:
+Ã¢ÂžÂ¢ Sales OF POS EDC Machine, SME Loan, Loan against electronic payment.
+Acquiring New Merchants And retaing existing Merchants.
+Ã¢ÂžÂ¢ Cold calling With CASA Team (ICICI BANK) Generating leads.
+Ã¢ÂžÂ¢  Field Visit Providing demo to Retailers shopkeeper SME &amp; Corporate merchant for Closing &amp; Signup.
+Worked with Mahal Pvt Ltd. as Sr. Sales Executive. (04th Mar 2016 to 03 Jan 2017)
+Nature of Work:
+Ã¢ÂžÂ¢ Calling on leads gegenerat Interacting with clients on call &amp; suggesting property Flat/Bunglows/N.A Plots &amp; Row houses as per their requirement.
+Ã¢ÂžÂ¢ Meeting new channel partners &amp; maintain relationship with channel partners for leads.
+Ã¢ÂžÂ¢ Achieving monthly targets, Maintaining reports &amp; updating seniors of daily activities.
+company - Bookmyflat.Com
+description - Arranging Site visit with client on lead generated
+Ã¢ÂžÂ¢  Closing deal by suggesting appropriate Residential property to clients as per their budget.</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>```json
+{
+    "summary": "The candidate's profile is primarily focused on Sales Management, real estate, and banking services. There is a significant mismatch between the candidate's professional background and the required expertise in Computer Science for AI training. While the candidate has basic technical skills like SQL, they lack the advanced Computer Science knowledge and technical writing experience required for this role.",
+    "match_score": 10,
+    "skill_match": {
+        "matched": [
+            "SQL",
+            "MS Office"
+        ],
+        "missing": [
+            "Advanced Computer Science domain knowledge",
+            "Technical writing",
+            "Complex problem-solving design",
+            "Academic content creation",
+            "Deep reasoning expertise"
+        ],
+        "score": 10
+    },
+    "experience_match": {
+        "matched_years": "0 (relevant to Computer Science)",
+        "required_years": "Subject Matter Expertise required",
+        "score": 0
+    },
+    "education_match": {
+        "matched_degree": "Bachelor's degree",
+        "required_degree": "Bachelor's or Master's in Computer Science",
+        "score": 20
+    },
+    "responsibility_match": {
+        "matched": [],
+        "missing": [
+            "Developing complex Q&amp;A pairs",
+            "Creating multi-step problem sets",
+            "Providing high-standard academic solutions",
+            "Collaborating on technical content refinement"
+        ],
+        "score": 0
+    },
+    "final_assessment": "Weak fit. The candidate's experience is entirely in Sales and Lead Generation, which does not align with the specialized Computer Science expertise required for this position."
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Requirements
+ Description and Requirements 
+Title: Data Partner - Computer Science
+Location: Asia - Remote
+Are you ready to use your domain knowledge to advance AI? Join us as a Data Partner and work remotely with flexible hours. We are seeking highly knowledgeable Subject Matter Expert to design advanced, domain-specific questions and solutions. The role involves creating challenging problem sets that test deep reasoning and expertise in the assigned field.
+Key Responsibilities:
+Develop complex, original question-and-answer pairs based on advanced topics in your area of expertise.
+Ensure questions involve multi-step problem-solving and critical thinking.
+Provide detailed, clear solutions that meet high academic standards.
+Collaborate with cross-functional teams to refine and enhance content.
+Basic Requirements:
+A completed master's degree, bachelor's degree, associate's degree or anything equivalent in Computer Science is essential
+Strong proficiency in English writing with excellent grammar, clarity, and the ability to explain complex concepts concisely
+Assessment:
+In order to be hired into the program, you’ll go through a subject-specific qualification exam that will determine your suitability for the position and complete ID verification.
+Payment:
+Currently, pay rates for experts range from $8 - $30 USD per hour
+Rates vary based on expertise, skills assessment, location, project need, and other factors. For example, higher rates may be offered to PhDs. Please review the payment terms for each project.
+Equal Opportunity:
+All qualified applicants will receive consideration for a contractual relationship without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, disability, or protected veteran status. At TELUS Digital AI, we are proud to offer equal opportunities and are committed to creating a diverse and inclusive community. All aspects of selection are based on applicants’ qualifications, merits, competence, and performance without regard to any characteristic related to diversity.
+Additional Job Description
+TELUS Digital AI Community
+Our global AI Community is a vibrant network of 1 million+ contributors from diverse backgrounds who help our customers collect, enhance, train, translate, and localize content to build better AI models. Become part of our growing community and make an impact supporting the machine learning models of some of the world’s largest brands.
+EEO Statement
+At TELUS International, we enable customer experience innovation through spirited teamwork, agile thinking, and a caring culture that puts customers first. TELUS International is the global arm of TELUS Corporation, one of the largest telecommunications service providers in Canada. We deliver contact center and business process outsourcing (BPO) solutions to some of the world's largest corporations in the consumer electronics, finance, telecommunications and utilities sectors. With global call center delivery capabilities, our multi-shore, multi-language programs offer safe, secure infrastructure, value-based pricing, skills-based resources and exceptional customer service - all backed by TELUS, our multi-billion dollar telecommunications parent.
+Equal Opportunity Employer
+At TELUS International, we are proud to be an equal opportunity employer and are committed to creating a diverse and inclusive workplace. All aspects of employment, including the decision to hire and promote, are based on applicants’ qualifications, merits, competence and performance without regard to any characteristic related to diversity.</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Education Details 
+January 1992 to January 2003 First year Science Mumbai, Maharashtra St micheal high
+Personal fitness trainer level3 
+personal trainer
+Skill Details 
+Company Details 
+company - Golds gym ,fitness solution,flora hotel
+description - Certification : american college of sports science golds gym heart saver reps level 3
+Responsibilities
+To obtain a challenging position which will commensurate with my qualification and experience in the field of health and fitness environment.
+Accomplishments
+Good
+Skills Used
+Fitness</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>```json
+{
+    "summary": "The candidate's profile is entirely unrelated to the job description. The resume describes a fitness professional/personal trainer, whereas the job requires a Subject Matter Expert in Computer Science.",
+    "match_score": 0,
+    "skill_match": {
+        "matched": [],
+        "missing": [
+            "Computer Science domain knowledge",
+            "Advanced problem-solving",
+            "Technical content creation",
+            "English writing proficiency for complex concepts",
+            "Critical thinking/reasoning design"
+        ],
+        "score": 0
+    },
+    "experience_match": {
+        "matched_years": "0",
+        "required_years": "Subject matter expertise in Computer Science required",
+        "score": 0
+    },
+    "education_match": {
+        "matched_degree": "First year Science",
+        "required_degree": "Bachelor's, Master's, or Associate's degree in Computer Science",
+        "score": 0
+    },
+    "responsibility_match": {
+        "matched": [],
+        "missing": [
+            "Developing complex question-and-answer pairs",
+            "Designing multi-step problem-solving tasks",
+            "Providing detailed academic solutions",
+            "Collaborating with cross-functional teams for content refinement"
+        ],
+        "score": 0
+    },
+    "final_assessment": "Weak fit. The candidate lacks the essential educational background and domain expertise in Computer Science required for this role."
+}
+```</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merged latest main branch
</commit_message>
<xml_diff>
--- a/data/dataset_complete(Data Scientist).xlsx
+++ b/data/dataset_complete(Data Scientist).xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14395,6 +14395,282 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Requirements
+ Description and Requirements 
+Title: Data Partner - Computer Science
+Location: Asia - Remote
+Are you ready to use your domain knowledge to advance AI? Join us as a Data Partner and work remotely with flexible hours. We are seeking highly knowledgeable Subject Matter Expert to design advanced, domain-specific questions and solutions. The role involves creating challenging problem sets that test deep reasoning and expertise in the assigned field.
+Key Responsibilities:
+Develop complex, original question-and-answer pairs based on advanced topics in your area of expertise.
+Ensure questions involve multi-step problem-solving and critical thinking.
+Provide detailed, clear solutions that meet high academic standards.
+Collaborate with cross-functional teams to refine and enhance content.
+Basic Requirements:
+A completed master's degree, bachelor's degree, associate's degree or anything equivalent in Computer Science is essential
+Strong proficiency in English writing with excellent grammar, clarity, and the ability to explain complex concepts concisely
+Assessment:
+In order to be hired into the program, you’ll go through a subject-specific qualification exam that will determine your suitability for the position and complete ID verification.
+Payment:
+Currently, pay rates for experts range from $8 - $30 USD per hour
+Rates vary based on expertise, skills assessment, location, project need, and other factors. For example, higher rates may be offered to PhDs. Please review the payment terms for each project.
+Equal Opportunity:
+All qualified applicants will receive consideration for a contractual relationship without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, disability, or protected veteran status. At TELUS Digital AI, we are proud to offer equal opportunities and are committed to creating a diverse and inclusive community. All aspects of selection are based on applicants’ qualifications, merits, competence, and performance without regard to any characteristic related to diversity.
+Additional Job Description
+TELUS Digital AI Community
+Our global AI Community is a vibrant network of 1 million+ contributors from diverse backgrounds who help our customers collect, enhance, train, translate, and localize content to build better AI models. Become part of our growing community and make an impact supporting the machine learning models of some of the world’s largest brands.
+EEO Statement
+At TELUS International, we enable customer experience innovation through spirited teamwork, agile thinking, and a caring culture that puts customers first. TELUS International is the global arm of TELUS Corporation, one of the largest telecommunications service providers in Canada. We deliver contact center and business process outsourcing (BPO) solutions to some of the world's largest corporations in the consumer electronics, finance, telecommunications and utilities sectors. With global call center delivery capabilities, our multi-shore, multi-language programs offer safe, secure infrastructure, value-based pricing, skills-based resources and exceptional customer service - all backed by TELUS, our multi-billion dollar telecommunications parent.
+Equal Opportunity Employer
+At TELUS International, we are proud to be an equal opportunity employer and are committed to creating a diverse and inclusive workplace. All aspects of employment, including the decision to hire and promote, are based on applicants’ qualifications, merits, competence and performance without regard to any characteristic related to diversity.</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Key Skills - Requirement Gathering - Requirement Analysis -Design Specifications - Client Communication - System Documentation - Problem solving - SDLC Operating Systems: Windows OS, UNIX (Linux/Ubuntu) Languages: Java, C++ Web Languages: JavaScript, HTML Tools: Citrix Software, System Architect, Quality Center v9.0 &amp; v10.0, Tortoise SVN, DOORS, Artifact Viewer, JformDesigner, JIRA, Microsoft D365 Other Skills: Microsoft Office, MS Excel, MS PowerPoint, MS Visio, AutoCAD, VLSI, MS-CIT Certified. Education Details 
+January 2012 BE Electronics Mumbai, Maharashtra Mumbai University
+January 2006    Maharashtra State Board
+Business Analyst 
+Business Analyst - Intertek India Pvt Ltd
+Skill Details 
+SDLC- Exprience - 75 months
+VISIO- Exprience - 60 months
+REQUIREMENT GATHERING- Exprience - 15 months
+Documentation- Exprience - Less than 1 year months
+Functional Testing- Exprience - Less than 1 year months
+Business Analysis- Exprience - Less than 1 year months
+Jira- Exprience - Less than 1 year monthsCompany Details 
+company - Intertek India Pvt Ltd
+description - Business Analyst. Key responsibilities include Requirements Gathering, Requirements Analysis. Documentation like FRD creation. Providing KT sessions to the team. Having Client Communication. Gap Analysis.
+company - Intertek India Pvt Ltd
+description - Requirement Gathering from Businesses. Creating FRDs.
+Ã¢ÂœÂ“ Vendor interaction for functional and technical disciplines.
+Ã¢ÂœÂ“ Creating Project Plan.
+Ã¢ÂœÂ“ Walkthrough to team regarding the requirement Ã¢ÂœÂ“ Change Proposal Management; Effort Estimation, Impact &amp; Gap Analysis Ã¢ÂœÂ“ Actively participate in Change proposal implementation &amp; testing and define ways for improvement / enhancement Ã¢ÂœÂ“ Defect analysis &amp; clarifying functional queries of team members &amp; developers Ã¢ÂœÂ“ Creating UAT Test cases. Executing the same.
+Ã¢ÂœÂ“ Test Management: Test Data creation, Test Case writing, Test Case Execution (Manual), Regression tests at various stages in the SDLC
+Project Details
+Project 1	Inlight (Feb 2018 till date)
+Platform	.Net
+Description:
+Inlight - (Supplier Risk Assessment Application)
+Inlight is an Application designed to assess the Suppliers within the Supply chain. The Application on boards the Importers, Exporters and Suppliers. Based on the role they perform a Questionnaire is assigned to them and they fill out the Questionnaire. Basis the answer a scoring methodology is defined and the Suppliers are assessed to be Critical, High, Medium and Low. This helps in assessing the risk involved in working with certain Suppliers in the Supply chain.
+Beyond Curriculum Ã¢ÂœÂ“ Completed Internship in L&amp;T Ã¢ÂœÂ“ Attended Logistics Business School Training in Germany.
+Ã¢ÂœÂ“ A1 Certified in German Language.
+Ã¢ÂœÂ“ Travelled Onsite for Business Meetings and Discussions with Clients.
+Personal Dossier .
+company - AllCargo India Pvt Ltd
+description - FRD creation
+Client communication
+Vendor Management
+Having product Walk through with the team.
+company - AllCargo India Pvt Ltd
+description - Requirement Gathering from Businesses. Creating BRDs and FSDs.
+Ã¢ÂœÂ“ Vendor interaction for functional and technical disciplines.
+Ã¢ÂœÂ“ Creating Project Plan.
+Ã¢ÂœÂ“ Analyzing business requirements and defining consistent, correct and complete specification Ã¢ÂœÂ“ Change Proposal Management; Effort Estimation, Impact &amp; Gap Analysis Ã¢ÂœÂ“ Actively participate in Change proposal implementation &amp; testing and define ways for improvement / enhancement Ã¢ÂœÂ“ Defect analysis &amp; clarifying functional queries of team members &amp; developers Ã¢ÂœÂ“ Prepare Requirement document, User manual, Test cases and training material Ã¢ÂœÂ“ Test Management: Test Data creation, Test Case writing, Test Case Execution (Manual), Regression tests at various stages in the SDLC
+Project Details
+Project 1	CRM (Nov 2017 to Feb 2018)
+Platform	Microsoft D365
+Description:
+CRM - (Sales Management System)
+CRM is a Software solution specially designed for handling Sales Management. This is a product provided by Microsoft which helps in tracking the sales of company, the activities of the salesperson, 360-degree view of customer accounts. This basically helps to get the overall status and view of various businesses the company is achieving from different Customers. A platform where the salesperson provides the details of Lead, Opportunity, Accounts and Businesses. Available on Cloud.
+Project 2	Credit Risk (Nov 2017 to Feb 2018)
+Platform	.Net
+Description:
+Credit Risk - (Customer credit check Management System)
+Credit Risk is a Software solution specially designed for checking the credit status of the customer from which businesses are gained. The software basically is designed to take the KYC and the consent from the customer. For those customers who provide the consent, the credit report and monitoring report are obtained from the Credit Bureau. Based on the reports the customer health can be determined and business with them can either be  or discontinued.
+Work Experience 3:
+company - Capgemini India Pvt Ltd
+description - Client: DB Schenker Ã¢ÂœÂ“ Analyzing business requirements and defining consistent, correct and complete specification Ã¢ÂœÂ“ Change Proposal Management; Effort Estimation, Impact &amp; Gap Analysis Ã¢ÂœÂ“ Actively participate in Change proposal implementation &amp; testing and define ways for improvement / enhancement Ã¢ÂœÂ“ Defect analysis &amp; clarifying functional queries of team members &amp; developers Ã¢ÂœÂ“ Prepare Requirement document, User manual, Test cases and training material Ã¢ÂœÂ“ Impart business process knowledge transfer to the team members. Prepare business / functional process workflow using Visio, UML etc Ã¢ÂœÂ“ Working knowledge of OOAD - Object Oriented Analysis &amp; Design concept.
+Ã¢ÂœÂ“ Helping the Junior BAs in their work. Supervising their work.
+Ã¢ÂœÂ“ Tools &amp; Applications: System Architect, DOORS, UML designs &amp; concepts, HP Quality Center, MWB, Jformdesigner Ã¢ÂœÂ“ Test Management: Test Data creation, Test Case writing, Test Case Execution (Manual), Regression tests at various stages in the SDLC
+Project Details
+company - Capgemini India Pvt Ltd
+description - Platform	Java
+Description:
+TANGO - (Sea &amp; Air Cargo Management System)
+TANGO is a Software solution specially designed for handling sea and air cargo (Import &amp; Export) Management. TANGO manages the creation of Shipment, Tracking the shipment via multiple service legs i.e. Pick-up, Delivery leg etc. It helps in managing the end to end shipment with respect to the entire department involvement (globally)
+Work Experience 2:
+company - Capgemini India Pvt Ltd
+description - </t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>```json
+{
+    "summary": "The candidate is an experienced Business Analyst with a solid technical foundation in software development lifecycles (SDLC) and programming languages such as Java and C++. However, there is a fundamental mismatch between the candidate's professional experience and the job requirements. The role demands an expert capable of designing complex, academic-level question-and-answer pairs for AI training, whereas the candidate's expertise lies in requirement gathering, functional documentation (FRD/BRD), and business process analysis.",
+    "match_score": 42,
+    "skill_match": {
+        "matched": [
+            "Java",
+            "C++",
+            "SDLC",
+            "Problem solving",
+            "Object Oriented Analysis &amp; Design",
+            "Technical Documentation",
+            "English proficiency (implied via documentation/communication tasks)"
+        ],
+        "missing": [
+            "AI model training/data generation",
+            "Advanced academic Q&amp;A design",
+            "Complex reasoning problem-set development",
+            "Subject Matter Expertise in pure Computer Science theory"
+        ],
+        "score": 45
+    },
+    "experience_match": {
+        "matched_years": "10+",
+        "required_years": "Not specified",
+        "score": 50
+    },
+    "education_match": {
+        "matched_degree": "BE Electronics",
+        "required_degree": "Bachelor's degree in Computer Science or equivalent",
+        "score": 90
+    },
+    "responsibility_match": {
+        "matched": [
+            "Analyzing complex requirements",
+            "Creating detailed documentation",
+            "Explaining concepts (via Knowledge Transfer sessions)",
+            "Problem solving"
+        ],
+        "missing": [
+            "Developing original complex question-and-answer pairs",
+            "Designing multi-step reasoning problem sets",
+            "Creating content specifically for AI model enhancement"
+        ],
+        "score": 30
+    },
+    "final_assessment": "Weak fit. While the candidate possesses a relevant technical degree and strong analytical and documentation skills, their career trajectory is focused on Business Analysis and Project Management rather than the academic/theoretical content creation required for this AI Data Partner role."
+}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Requirements
+ Description and Requirements 
+Title: Data Partner - Computer Science
+Location: Asia - Remote
+Are you ready to use your domain knowledge to advance AI? Join us as a Data Partner and work remotely with flexible hours. We are seeking highly knowledgeable Subject Matter Expert to design advanced, domain-specific questions and solutions. The role involves creating challenging problem sets that test deep reasoning and expertise in the assigned field.
+Key Responsibilities:
+Develop complex, original question-and-answer pairs based on advanced topics in your area of expertise.
+Ensure questions involve multi-step problem-solving and critical thinking.
+Provide detailed, clear solutions that meet high academic standards.
+Collaborate with cross-functional teams to refine and enhance content.
+Basic Requirements:
+A completed master's degree, bachelor's degree, associate's degree or anything equivalent in Computer Science is essential
+Strong proficiency in English writing with excellent grammar, clarity, and the ability to explain complex concepts concisely
+Assessment:
+In order to be hired into the program, you’ll go through a subject-specific qualification exam that will determine your suitability for the position and complete ID verification.
+Payment:
+Currently, pay rates for experts range from $8 - $30 USD per hour
+Rates vary based on expertise, skills assessment, location, project need, and other factors. For example, higher rates may be offered to PhDs. Please review the payment terms for each project.
+Equal Opportunity:
+All qualified applicants will receive consideration for a contractual relationship without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, disability, or protected veteran status. At TELUS Digital AI, we are proud to offer equal opportunities and are committed to creating a diverse and inclusive community. All aspects of selection are based on applicants’ qualifications, merits, competence, and performance without regard to any characteristic related to diversity.
+Additional Job Description
+TELUS Digital AI Community
+Our global AI Community is a vibrant network of 1 million+ contributors from diverse backgrounds who help our customers collect, enhance, train, translate, and localize content to build better AI models. Become part of our growing community and make an impact supporting the machine learning models of some of the world’s largest brands.
+EEO Statement
+At TELUS International, we enable customer experience innovation through spirited teamwork, agile thinking, and a caring culture that puts customers first. TELUS International is the global arm of TELUS Corporation, one of the largest telecommunications service providers in Canada. We deliver contact center and business process outsourcing (BPO) solutions to some of the world's largest corporations in the consumer electronics, finance, telecommunications and utilities sectors. With global call center delivery capabilities, our multi-shore, multi-language programs offer safe, secure infrastructure, value-based pricing, skills-based resources and exceptional customer service - all backed by TELUS, our multi-billion dollar telecommunications parent.
+Equal Opportunity Employer
+At TELUS International, we are proud to be an equal opportunity employer and are committed to creating a diverse and inclusive workplace. All aspects of employment, including the decision to hire and promote, are based on applicants’ qualifications, merits, competence and performance without regard to any characteristic related to diversity.</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Ã¢Â€Â¢ Achievement oriented with people management skills and an ability to manage change with ease. Ã¢Â€Â¢ Proven strength in problem solving, coordination and analysis. Ã¢Â€Â¢ Strong communication, interpersonal, learning and organizing skills matched with the ability to manage stress, time and people effectively. Ã¢Â€Â¢ Able to handle multiple task &amp; projects simultaneously. Ã¢Â€Â¢ Willing to travel &amp; relocate.Education Details 
+ B.E Electrical and Electronics Engineering Gulbarga, Karnataka VTU (Vishweshwariya University)
+ HSC  Wai, Maharashtra Kisanveer Mahavidyalay WAI
+    Kohlapur University
+Electrical Engineer 
+Electrical Engineer - REFCON ENGINEERING PVT. LTD
+Skill Details 
+Company Details 
+company - REFCON ENGINEERING PVT. LTD
+description - GREENFIELD PROJECT: -		Project Status 
+1) LIBS Braseries, Burkena Faso (Africa)		Completed 2) Citrus Processing India, Nanded		Completed 3) Carlsberg Group, Myanmar (Yangon)		Completed 4) U.B (United Breweries), Mysore.		Completed 5) U.B (United Breweries), Hyderabad.		Completed 6) Haldiram Foods Pvt. Ltd. Nagpur		Completed 7) Tetra-Pak India Pvt. Ltd. Amreli		Completed 8) U.B (United Breweries), Rajasthan		Completed Ã¢ÂÂ– Handling Activities in Project: - 
+Ã¢ÂžÂ¢ Preparing project schedules / plans, engineering designs / drawings and technical specifications as per clients' requirements.
+Ã¢ÂžÂ¢ Review on Process P&amp;ID's for Selection of Instrument to get Energy efficient process with Material Specifications. Approval &amp; modifications of Electrical drawing as per requirement of Process Flow diagrams &amp; General Electrical Standards.
+Ã¢ÂžÂ¢ Carry out Automation Engineering which includes hardware and software specification, Generate control philosophy for process automation as per P&amp;ID process. Necessary technical documentation, O&amp;M manuals.
+Ã¢ÂžÂ¢ Calculate the Estimation value of projects for price bidding with clients includes MCC &amp; PLC panel, power &amp; control cabling, trays &amp; earthing material Etc.
+Ã¢ÂžÂ¢ Selection of Electrical Switchgear for HT, LT, PCC, MCC, APFC Panels, Power &amp; Control cable, Motors, Protection &amp; metering CT &amp; PTs, ACBs, Earthing, lightning, Analog &amp; Digital Instruments.
+Ã¢ÂžÂ¢ Floating project enquiries &amp; communicate with Vendors, Evaluate Vendor quotes for Technical Alignment.
+Ã¢ÂžÂ¢ Generate Power distribution SLD drawings as per the load flow, General arrangement drawings for panels, Controllers logic diagrams, Developing of Cable route plan and schedules, Cable Tray layout on AutoCAD tool with detailing.
+Ã¢ÂžÂ¢ Installation, Commissioning &amp; Troubleshooting of MCC, PLC &amp; LT panels, VFD Drives, Soft-Starters, Programming of Danfoss, Schnider, Vacon, Siemens, ABB Drives.
+Ã¢ÂžÂ¢ Working experience on Siemens S7-300, 1200, 1500, Et-200S Series &amp; Allen-bready RS-Logix5000 PLC.
+Ã¢ÂžÂ¢ Installation, Calibration &amp; Troubleshooting of field Instruments as Pressure &amp; Temperature Transmitter, Pneumatic valves, Actuators, Modulating valves, Solenoid valve, flow meter &amp; flow switches, Flow Transmitter, Level Transmitter etc. Carry out Loop testing as per control cable schedule, Ã¢ÂžÂ¢ Hands on experience in Troubleshooting, Engineering Services and Maintenance &amp; Operation &amp; managing of various electrical power system equipments. Supervising commissioning activities.
+Ã¢ÂžÂ¢ Handling Mechanical Maintenance &amp; Service activities in operating plant.
+company - KISANVEER SUGARS PVT. LTD
+description - Handling Activities: - 
+Ã¢ÂžÂ¢ With over 1.5 years of experience worked as Asst. Electrical Engineer from ERECTION FIELD across 22 MW Power Plant for Testing and Commissioning, Electrical Maintenance, Operation, and allied activities.
+Ã¢ÂžÂ¢ Testing, Commissioning &amp; installation of HT &amp; LT panels, VFD drives &amp; DC drives Panels.
+Ã¢ÂžÂ¢ Scheduling and planning predictive, preventive maintenance for process plants, and root cause analysis including budgeting and cost control activities.
+Ã¢ÂžÂ¢ Managing Overhauling and maintenance of LT Motors &amp; DC Shunt Motors, Panel Switchgears, VFDs &amp; soft starters, DG Set with AMF panel &amp; Plant Lighting.
+Ã¢ÂžÂ¢ Installation, commissioning &amp; Maintenance of Power &amp; Distribution Transformer, ACB, VCB, SF6 Breaker, CT &amp; PT units, FCBC Panels, UPS, Ã¢ÂžÂ¢ Protection system include Microprocessor based relay, Numerical relay with relay co-ordination.
+Ã¢ÂžÂ¢ Monitoring plans/schedules to start maintenance activities &amp; achieving targets and implementing maintenance systems During Shut down Time.
+Ã¢ÂžÂ¢ Daily Power monitoring, calculations and reporting on monthly basis.</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>```json
+{
+    "summary": "The candidate is a highly skilled Electrical Engineer with significant experience in automation, power systems, and technical documentation. However, there is a fundamental domain mismatch as the job description specifically requires Subject Matter Expertise in Computer Science, whereas the candidate's expertise lies in Electrical and Electronics Engineering.",
+    "match_score": 5,
+    "skill_match": {
+        "matched": [
+            "Problem solving",
+            "Technical documentation",
+            "Analysis",
+            "Communication"
+        ],
+        "missing": [
+            "Computer Science expertise",
+            "Algorithms",
+            "Data Structures",
+            "Software Engineering",
+            "AI model training methodology",
+            "Advanced academic writing in CS"
+        ],
+        "score": 10
+    },
+    "experience_match": {
+        "matched_years": "0 years in Computer Science",
+        "required_years": "Not specified (Domain expertise required)",
+        "score": 0
+    },
+    "education_match": {
+        "matched_degree": [
+            "B.E. Electrical and Electronics Engineering"
+        ],
+        "required_degree": [
+            "Bachelor's, Master's, or Associate's degree in Computer Science"
+        ],
+        "score": 0
+    },
+    "responsibility_match": {
+        "matched": [],
+        "missing": [
+            "Develop complex, original question-and-answer pairs in Computer Science",
+            "Design advanced, domain-specific questions for AI training",
+            "Create multi-step problem-solving sets",
+            "Provide detailed solutions meeting high academic standards"
+        ],
+        "score": 0
+    },
+    "final_assessment": "Weak fit. While the candidate is an accomplished professional in the electrical engineering field, they lack the required Computer Science background and the specific content creation experience necessary for this role."
+}
+```</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>